<commit_message>
Add note createTime tests and reorganize order cases into note directory
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/云下/bom.xlsx
+++ b/excel/云下/bom.xlsx
@@ -7,13 +7,14 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId3"/>
+    <sheet name="导入注意" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="253">
   <si>
     <t/>
   </si>
@@ -718,6 +719,60 @@
   </si>
   <si>
     <t>片</t>
+  </si>
+  <si>
+    <t>1、每个bom必须有单位</t>
+  </si>
+  <si>
+    <t>2、保持餐品名称不要变，否则可能会新增餐品（）</t>
+  </si>
+  <si>
+    <t>2、保持餐品名称不要变，否则可能会新增餐品（加了餐品编码能识别到不会新增餐品）</t>
+  </si>
+  <si>
+    <t>3、如果对应物料不存在，先建立物料，或者在云下物料</t>
+  </si>
+  <si>
+    <t>3、如果对应物料不存在，先建立物料，或者在“云下物料”新增记录重新导物料</t>
+  </si>
+  <si>
+    <t>4、产品</t>
+  </si>
+  <si>
+    <t>1、每个bom必须有单位，并且单位必须在物料规格中存在。</t>
+  </si>
+  <si>
+    <t>4、物料的数量和单位不要写在同一个格子里面，分开写，否则会识别错误。</t>
+  </si>
+  <si>
+    <t>云下冰芒生椰米布  x  好运椰</t>
+  </si>
+  <si>
+    <t>云下冰芒生椰米布X好运椰</t>
+  </si>
+  <si>
+    <t>酸萝卜牛肉锅（1～2人份）</t>
+  </si>
+  <si>
+    <t>M020</t>
+  </si>
+  <si>
+    <t>外卖酸萝卜牛肉锅</t>
+  </si>
+  <si>
+    <t>赠送酸木瓜水</t>
+  </si>
+  <si>
+    <t>GOO9</t>
+  </si>
+  <si>
+    <t>G009</t>
+  </si>
+  <si>
+    <t>雪域青稞粑粑  |  桂花香</t>
+  </si>
+  <si>
+    <t>青稞小米饼</t>
   </si>
 </sst>
 </file>
@@ -727,7 +782,7 @@
   <numFmts count="1">
     <numFmt numFmtId="300" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <sz val="11"/>
@@ -750,11 +805,14 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <color rgb="FFFF0000"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -762,6 +820,9 @@
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="none">
@@ -786,9 +847,9 @@
     </border>
   </borders>
   <cellStyleXfs>
-    <xf numFmtId="300" fontId="4" fillId="2" borderId="1" xfId="0"/>
+    <xf numFmtId="300" fontId="5" fillId="3" borderId="1" xfId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -799,8 +860,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="300" fontId="4" fillId="2" borderId="1" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="300" fontId="5" fillId="3" borderId="1" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf fontId="4" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1131,7 +1195,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr/>
-  <dimension ref="F367"/>
+  <dimension ref="F385"/>
+  <cols>
+    <col min="2" max="2" width="23.4219" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
@@ -2673,8 +2740,8 @@
       <c r="A106" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B106" s="4" t="s">
-        <v>95</v>
+      <c r="B106" s="7" t="s">
+        <v>244</v>
       </c>
       <c r="C106" s="4" t="s">
         <v>96</v>
@@ -5669,8 +5736,8 @@
       <c r="E311" s="4">
         <v>100</v>
       </c>
-      <c r="F311" s="4" t="s">
-        <v>21</v>
+      <c r="F311" s="5" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="312" spans="1:6">
@@ -6527,6 +6594,292 @@
       </c>
       <c r="F367" s="4" t="s">
         <v>93</v>
+      </c>
+    </row>
+    <row r="368" spans="1:6">
+      <c r="A368" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="B368" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="C368" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D368" s="4">
+        <v>1003004</v>
+      </c>
+      <c r="E368" s="8">
+        <v>276</v>
+      </c>
+      <c r="F368" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="369" spans="1:6">
+      <c r="A369" s="4" t="s"/>
+      <c r="B369" s="4" t="s"/>
+      <c r="C369" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="D369" s="4">
+        <v>1009010</v>
+      </c>
+      <c r="E369" s="8">
+        <v>125</v>
+      </c>
+      <c r="F369" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="370" spans="1:6">
+      <c r="A370" s="4" t="s"/>
+      <c r="B370" s="4" t="s"/>
+      <c r="C370" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="D370" s="4">
+        <v>1006043</v>
+      </c>
+      <c r="E370" s="8">
+        <v>143</v>
+      </c>
+      <c r="F370" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="371" spans="1:6">
+      <c r="A371" s="4" t="s"/>
+      <c r="B371" s="4" t="s"/>
+      <c r="C371" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D371" s="4">
+        <v>1006056</v>
+      </c>
+      <c r="E371" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="F371" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="372" spans="1:6">
+      <c r="A372" s="4" t="s"/>
+      <c r="B372" s="4" t="s"/>
+      <c r="C372" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D372" s="4">
+        <v>1006027</v>
+      </c>
+      <c r="E372" s="4">
+        <v>10.4</v>
+      </c>
+      <c r="F372" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="373" spans="1:6">
+      <c r="A373" s="4" t="s"/>
+      <c r="B373" s="4" t="s"/>
+      <c r="C373" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D373" s="4">
+        <v>1001002</v>
+      </c>
+      <c r="E373" s="4">
+        <v>12</v>
+      </c>
+      <c r="F373" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="374" spans="1:6">
+      <c r="A374" s="4" t="s"/>
+      <c r="B374" s="4" t="s"/>
+      <c r="C374" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D374" s="4">
+        <v>1001004</v>
+      </c>
+      <c r="E374" s="4">
+        <v>6.2</v>
+      </c>
+      <c r="F374" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="375" spans="1:6">
+      <c r="A375" s="4" t="s"/>
+      <c r="B375" s="4" t="s"/>
+      <c r="C375" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="D375" s="4">
+        <v>1006003</v>
+      </c>
+      <c r="E375" s="4">
+        <v>0.3</v>
+      </c>
+      <c r="F375" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="376" spans="1:6">
+      <c r="A376" s="4" t="s"/>
+      <c r="B376" s="4" t="s"/>
+      <c r="C376" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="D376" s="4">
+        <v>1006010</v>
+      </c>
+      <c r="E376" s="4">
+        <v>0.42</v>
+      </c>
+      <c r="F376" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="377" spans="1:6">
+      <c r="A377" s="4" t="s"/>
+      <c r="B377" s="4" t="s"/>
+      <c r="C377" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D377" s="4">
+        <v>1006014</v>
+      </c>
+      <c r="E377" s="4">
+        <v>12.62</v>
+      </c>
+      <c r="F377" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="378" spans="1:6">
+      <c r="A378" s="4" t="s"/>
+      <c r="B378" s="4" t="s"/>
+      <c r="C378" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D378" s="4">
+        <v>1006009</v>
+      </c>
+      <c r="E378" s="4">
+        <v>1</v>
+      </c>
+      <c r="F378" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="379" spans="3:6">
+      <c r="C379" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D379" s="4">
+        <v>1001010</v>
+      </c>
+      <c r="E379" s="4">
+        <v>2</v>
+      </c>
+      <c r="F379" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="380" spans="3:6">
+      <c r="C380" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D380" s="4">
+        <v>1005004</v>
+      </c>
+      <c r="E380" s="4">
+        <v>50</v>
+      </c>
+      <c r="F380" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="381" spans="3:6">
+      <c r="C381" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D381" s="4">
+        <v>1006022</v>
+      </c>
+      <c r="E381">
+        <v>4</v>
+      </c>
+      <c r="F381" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="382" spans="3:6">
+      <c r="C382" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D382" s="4">
+        <v>1006028</v>
+      </c>
+      <c r="E382">
+        <v>10</v>
+      </c>
+      <c r="F382" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="383" spans="3:6">
+      <c r="C383" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D383" s="4">
+        <v>1006048</v>
+      </c>
+      <c r="E383">
+        <v>50</v>
+      </c>
+      <c r="F383" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="384" spans="1:6">
+      <c r="A384" t="s">
+        <v>250</v>
+      </c>
+      <c r="B384" t="s">
+        <v>248</v>
+      </c>
+      <c r="C384" t="s">
+        <v>85</v>
+      </c>
+      <c r="D384">
+        <v>1007013</v>
+      </c>
+      <c r="E384">
+        <f>=400/16</f>
+        <v>25</v>
+      </c>
+      <c r="F384" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="385" spans="3:6">
+      <c r="C385" t="s">
+        <v>202</v>
+      </c>
+      <c r="D385" s="4">
+        <v>1007005</v>
+      </c>
+      <c r="E385">
+        <f>=350/16</f>
+        <v>21.875</v>
+      </c>
+      <c r="F385" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -6974,7 +7327,6 @@
     <ignoredError sqref="E105" numberStoredAsText="1"/>
     <ignoredError sqref="F105" numberStoredAsText="1"/>
     <ignoredError sqref="A106" numberStoredAsText="1"/>
-    <ignoredError sqref="B106" numberStoredAsText="1"/>
     <ignoredError sqref="C106" numberStoredAsText="1"/>
     <ignoredError sqref="D106" numberStoredAsText="1"/>
     <ignoredError sqref="E106" numberStoredAsText="1"/>
@@ -7833,7 +8185,6 @@
     <ignoredError sqref="C311" numberStoredAsText="1"/>
     <ignoredError sqref="D311" numberStoredAsText="1"/>
     <ignoredError sqref="E311" numberStoredAsText="1"/>
-    <ignoredError sqref="F311" numberStoredAsText="1"/>
     <ignoredError sqref="A312" numberStoredAsText="1"/>
     <ignoredError sqref="B312" numberStoredAsText="1"/>
     <ignoredError sqref="C312" numberStoredAsText="1"/>
@@ -7849,7 +8200,6 @@
     <ignoredError sqref="E314" numberStoredAsText="1"/>
     <ignoredError sqref="F314" numberStoredAsText="1"/>
     <ignoredError sqref="C315" numberStoredAsText="1"/>
-    <ignoredError sqref="D315" numberStoredAsText="1"/>
     <ignoredError sqref="E315" numberStoredAsText="1"/>
     <ignoredError sqref="F315" numberStoredAsText="1"/>
     <ignoredError sqref="A316" numberStoredAsText="1"/>
@@ -8084,4 +8434,36 @@
     <ignoredError sqref="F367" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName="导入注意">
+    <tabColor/>
+  </sheetPr>
+  <dimension ref="B5"/>
+  <sheetFormatPr baseColWidth="13" defaultRowHeight="18" customHeight="1"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="6" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2">
+      <c r="B3" s="6" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2">
+      <c r="B4" s="6" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2">
+      <c r="B5" s="6" t="s">
+        <v>242</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>